<commit_message>
Update Hawaii Excel datasets [auto]
</commit_message>
<xml_diff>
--- a/Paper1/Paper/Data/HawaiiData.xlsx
+++ b/Paper1/Paper/Data/HawaiiData.xlsx
@@ -531,7 +531,7 @@
         <v>6.87323</v>
       </c>
       <c r="K2" t="n">
-        <v>2.30506</v>
+        <v>2.30536</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -574,7 +574,7 @@
         <v>4.15367</v>
       </c>
       <c r="K3" t="n">
-        <v>2.43806</v>
+        <v>2.42488</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -617,7 +617,7 @@
         <v>7.55398</v>
       </c>
       <c r="K4" t="n">
-        <v>2.13186</v>
+        <v>2.13214</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -660,7 +660,7 @@
         <v>0.74259</v>
       </c>
       <c r="K5" t="n">
-        <v>2.02259</v>
+        <v>2.02286</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         <v>1.77784</v>
       </c>
       <c r="K6" t="n">
-        <v>1.97981</v>
+        <v>1.98007</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -746,7 +746,7 @@
         <v>2.02157</v>
       </c>
       <c r="K7" t="n">
-        <v>1.71466</v>
+        <v>1.71488</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -789,7 +789,7 @@
         <v>4.61385</v>
       </c>
       <c r="K8" t="n">
-        <v>1.47327</v>
+        <v>1.47346</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -832,7 +832,7 @@
         <v>7.05482</v>
       </c>
       <c r="K9" t="n">
-        <v>1.21046</v>
+        <v>1.21062</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -875,7 +875,7 @@
         <v>8.03481</v>
       </c>
       <c r="K10" t="n">
-        <v>0.70021</v>
+        <v>0.7003</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -918,7 +918,7 @@
         <v>5.90081</v>
       </c>
       <c r="K11" t="n">
-        <v>0.34933</v>
+        <v>0.34938</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -1004,7 +1004,7 @@
         <v>3.56805</v>
       </c>
       <c r="K13" t="n">
-        <v>-0.19352</v>
+        <v>-0.19355</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -1047,7 +1047,7 @@
         <v>2.00281</v>
       </c>
       <c r="K14" t="n">
-        <v>-0.7725</v>
+        <v>-0.7726</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
         <v>3.20213</v>
       </c>
       <c r="K15" t="n">
-        <v>-1.00347</v>
+        <v>-1.0036</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -1133,7 +1133,7 @@
         <v>4.71972</v>
       </c>
       <c r="K16" t="n">
-        <v>-1.21118</v>
+        <v>-1.21134</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -1176,7 +1176,7 @@
         <v>5.26354</v>
       </c>
       <c r="K17" t="n">
-        <v>-1.68641</v>
+        <v>-1.68662</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -1219,7 +1219,7 @@
         <v>4.22933</v>
       </c>
       <c r="K18" t="n">
-        <v>-1.97994</v>
+        <v>-1.9802</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -1262,7 +1262,7 @@
         <v>3.76165</v>
       </c>
       <c r="K19" t="n">
-        <v>-2.26483</v>
+        <v>-2.26512</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -1305,7 +1305,7 @@
         <v>0.94789</v>
       </c>
       <c r="K20" t="n">
-        <v>-2.53116</v>
+        <v>-2.53148</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
         <v>-1.13358</v>
       </c>
       <c r="K21" t="n">
-        <v>-2.58488</v>
+        <v>-2.58521</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -1391,7 +1391,7 @@
         <v>-2.8686</v>
       </c>
       <c r="K22" t="n">
-        <v>-2.39506</v>
+        <v>-2.39536</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
         <v>-2.60379</v>
       </c>
       <c r="K23" t="n">
-        <v>-2.39814</v>
+        <v>-2.39845</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -1477,7 +1477,7 @@
         <v>-2.90647</v>
       </c>
       <c r="K24" t="n">
-        <v>-2.19468</v>
+        <v>-2.18205</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -1520,7 +1520,7 @@
         <v>-3.72218</v>
       </c>
       <c r="K25" t="n">
-        <v>-1.93899</v>
+        <v>-1.93924</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -1563,7 +1563,7 @@
         <v>-6.68686</v>
       </c>
       <c r="K26" t="n">
-        <v>-1.50513</v>
+        <v>-1.50532</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -1606,7 +1606,7 @@
         <v>-7.29507</v>
       </c>
       <c r="K27" t="n">
-        <v>-0.97466</v>
+        <v>-0.97479</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -1649,7 +1649,7 @@
         <v>-7.18887</v>
       </c>
       <c r="K28" t="n">
-        <v>-0.46954</v>
+        <v>-0.46961</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -1692,7 +1692,7 @@
         <v>-8.49579</v>
       </c>
       <c r="K29" t="n">
-        <v>0.31426</v>
+        <v>0.3143</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -1735,7 +1735,7 @@
         <v>-7.96439</v>
       </c>
       <c r="K30" t="n">
-        <v>0.61647</v>
+        <v>0.62967</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -1778,7 +1778,7 @@
         <v>-7.24745</v>
       </c>
       <c r="K31" t="n">
-        <v>1.11916</v>
+        <v>1.1193</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -1821,7 +1821,7 @@
         <v>-7.5816</v>
       </c>
       <c r="K32" t="n">
-        <v>1.3314</v>
+        <v>1.33158</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -1864,7 +1864,7 @@
         <v>-8.440099999999999</v>
       </c>
       <c r="K33" t="n">
-        <v>1.54455</v>
+        <v>1.55796</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -1907,7 +1907,7 @@
         <v>-7.62422</v>
       </c>
       <c r="K34" t="n">
-        <v>1.56992</v>
+        <v>1.57013</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -1950,7 +1950,7 @@
         <v>-5.89477</v>
       </c>
       <c r="K35" t="n">
-        <v>1.61162</v>
+        <v>1.61184</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -1993,7 +1993,7 @@
         <v>-7.24322</v>
       </c>
       <c r="K36" t="n">
-        <v>1.34636</v>
+        <v>1.33316</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -2036,7 +2036,7 @@
         <v>-7.38131</v>
       </c>
       <c r="K37" t="n">
-        <v>1.02821</v>
+        <v>1.04153</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -2079,7 +2079,7 @@
         <v>-3.30781</v>
       </c>
       <c r="K38" t="n">
-        <v>0.5928099999999999</v>
+        <v>0.59289</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -2122,7 +2122,7 @@
         <v>-2.16373</v>
       </c>
       <c r="K39" t="n">
-        <v>0.03937</v>
+        <v>0.03938</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -2165,7 +2165,7 @@
         <v>-1.56239</v>
       </c>
       <c r="K40" t="n">
-        <v>-0.23588</v>
+        <v>-0.23591</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
         <v>-0.60228</v>
       </c>
       <c r="K41" t="n">
-        <v>-0.75708</v>
+        <v>-0.75718</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -2251,7 +2251,7 @@
         <v>-1.01636</v>
       </c>
       <c r="K42" t="n">
-        <v>-1.082</v>
+        <v>-1.09503</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
@@ -2294,7 +2294,7 @@
         <v>-1.00361</v>
       </c>
       <c r="K43" t="n">
-        <v>-1.06771</v>
+        <v>-1.06785</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -2337,7 +2337,7 @@
         <v>1.32015</v>
       </c>
       <c r="K44" t="n">
-        <v>-1.27488</v>
+        <v>-1.27505</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
@@ -2380,7 +2380,7 @@
         <v>0.68588</v>
       </c>
       <c r="K45" t="n">
-        <v>-1.24805</v>
+        <v>-1.26105</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
         <v>1.35223</v>
       </c>
       <c r="K46" t="n">
-        <v>-1.22094</v>
+        <v>-1.2211</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
@@ -2466,7 +2466,7 @@
         <v>1.09793</v>
       </c>
       <c r="K47" t="n">
-        <v>-1.00104</v>
+        <v>-0.98817</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -2509,7 +2509,7 @@
         <v>2.6756</v>
       </c>
       <c r="K48" t="n">
-        <v>-0.4298</v>
+        <v>-0.42986</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
@@ -2552,7 +2552,7 @@
         <v>2.51899</v>
       </c>
       <c r="K49" t="n">
-        <v>0.11743</v>
+        <v>0.10438</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
@@ -2595,7 +2595,7 @@
         <v>1.41031</v>
       </c>
       <c r="K50" t="n">
-        <v>0.60241</v>
+        <v>0.61559</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
@@ -2638,7 +2638,7 @@
         <v>0.18329</v>
       </c>
       <c r="K51" t="n">
-        <v>0.87892</v>
+        <v>0.89215</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -2681,7 +2681,7 @@
         <v>-0.83586</v>
       </c>
       <c r="K52" t="n">
-        <v>0.88007</v>
+        <v>0.88019</v>
       </c>
       <c r="L52" t="inlineStr">
         <is>
@@ -2724,7 +2724,7 @@
         <v>-0.6408700000000001</v>
       </c>
       <c r="K53" t="n">
-        <v>0.84177</v>
+        <v>0.84188</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
@@ -2767,7 +2767,7 @@
         <v>-0.46422</v>
       </c>
       <c r="K54" t="n">
-        <v>0.88297</v>
+        <v>0.88309</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
@@ -2810,7 +2810,7 @@
         <v>-1.2576</v>
       </c>
       <c r="K55" t="n">
-        <v>0.61858</v>
+        <v>0.6186700000000001</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
@@ -2853,7 +2853,7 @@
         <v>-2.05585</v>
       </c>
       <c r="K56" t="n">
-        <v>0.57979</v>
+        <v>0.57986</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
@@ -2896,7 +2896,7 @@
         <v>-0.07042</v>
       </c>
       <c r="K57" t="n">
-        <v>0.30279</v>
+        <v>0.30283</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
@@ -2939,7 +2939,7 @@
         <v>-0.9904500000000001</v>
       </c>
       <c r="K58" t="n">
-        <v>0.24984</v>
+        <v>0.26302</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
@@ -3025,7 +3025,7 @@
         <v>-1.08805</v>
       </c>
       <c r="K60" t="n">
-        <v>-0.30085</v>
+        <v>-0.28781</v>
       </c>
       <c r="L60" t="inlineStr">
         <is>
@@ -3068,7 +3068,7 @@
         <v>-1.03275</v>
       </c>
       <c r="K61" t="n">
-        <v>-0.5734399999999999</v>
+        <v>-0.56048</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         <v>1.93804</v>
       </c>
       <c r="K64" t="n">
-        <v>-0.52083</v>
+        <v>-0.5209</v>
       </c>
       <c r="L64" t="inlineStr">
         <is>
@@ -3240,7 +3240,7 @@
         <v>0.72118</v>
       </c>
       <c r="K65" t="n">
-        <v>-0.28694</v>
+        <v>-0.28698</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
@@ -3283,7 +3283,7 @@
         <v>1.0878</v>
       </c>
       <c r="K66" t="n">
-        <v>-0.01306</v>
+        <v>0</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
@@ -3326,7 +3326,7 @@
         <v>2.17111</v>
       </c>
       <c r="K67" t="n">
-        <v>0.23545</v>
+        <v>0.23548</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
@@ -3369,7 +3369,7 @@
         <v>2.45751</v>
       </c>
       <c r="K68" t="n">
-        <v>0.79916</v>
+        <v>0.79927</v>
       </c>
       <c r="L68" t="inlineStr">
         <is>
@@ -3412,7 +3412,7 @@
         <v>2.30566</v>
       </c>
       <c r="K69" t="n">
-        <v>1.11563</v>
+        <v>1.11578</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
         <v>3.13813</v>
       </c>
       <c r="K71" t="n">
-        <v>1.15577</v>
+        <v>1.14263</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
@@ -3541,7 +3541,7 @@
         <v>2.07499</v>
       </c>
       <c r="K72" t="n">
-        <v>0.91839</v>
+        <v>0.90527</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
@@ -3584,7 +3584,7 @@
         <v>3.72548</v>
       </c>
       <c r="K73" t="n">
-        <v>0.95688</v>
+        <v>0.94377</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -3670,7 +3670,7 @@
         <v>1.52746</v>
       </c>
       <c r="K75" t="n">
-        <v>0.93042</v>
+        <v>0.91731</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -3713,7 +3713,7 @@
         <v>1.24683</v>
       </c>
       <c r="K76" t="n">
-        <v>0.92932</v>
+        <v>0.94253</v>
       </c>
       <c r="L76" t="inlineStr">
         <is>
@@ -3756,7 +3756,7 @@
         <v>1.24298</v>
       </c>
       <c r="K77" t="n">
-        <v>0.96795</v>
+        <v>0.98116</v>
       </c>
       <c r="L77" t="inlineStr">
         <is>
@@ -3799,7 +3799,7 @@
         <v>-0.03912</v>
       </c>
       <c r="K78" t="n">
-        <v>1.21505</v>
+        <v>1.20199</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
@@ -3842,7 +3842,7 @@
         <v>-1.36338</v>
       </c>
       <c r="K79" t="n">
-        <v>1.22667</v>
+        <v>1.22683</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -3885,7 +3885,7 @@
         <v>-1.24423</v>
       </c>
       <c r="K80" t="n">
-        <v>0.93579</v>
+        <v>0.93592</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
@@ -3928,7 +3928,7 @@
         <v>-1.38608</v>
       </c>
       <c r="K81" t="n">
-        <v>1.19418</v>
+        <v>1.20732</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
@@ -4014,7 +4014,7 @@
         <v>-1.15059</v>
       </c>
       <c r="K83" t="n">
-        <v>1.71384</v>
+        <v>1.72705</v>
       </c>
       <c r="L83" t="inlineStr">
         <is>
@@ -4057,7 +4057,7 @@
         <v>-1.29216</v>
       </c>
       <c r="K84" t="n">
-        <v>2.22309</v>
+        <v>2.22338</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
@@ -4100,7 +4100,7 @@
         <v>-2.01288</v>
       </c>
       <c r="K85" t="n">
-        <v>2.2202</v>
+        <v>2.23348</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
@@ -4186,7 +4186,7 @@
         <v>-1.27068</v>
       </c>
       <c r="K87" t="n">
-        <v>2.46689</v>
+        <v>2.46721</v>
       </c>
       <c r="L87" t="inlineStr">
         <is>
@@ -4272,7 +4272,7 @@
         <v>-0.57021</v>
       </c>
       <c r="K89" t="n">
-        <v>2.50032</v>
+        <v>2.48737</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -4315,7 +4315,7 @@
         <v>0.17421</v>
       </c>
       <c r="K90" t="n">
-        <v>2.01368</v>
+        <v>2.02685</v>
       </c>
       <c r="L90" t="inlineStr">
         <is>
@@ -4358,7 +4358,7 @@
         <v>0.38878</v>
       </c>
       <c r="K91" t="n">
-        <v>1.97241</v>
+        <v>1.97267</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -4401,7 +4401,7 @@
         <v>-0.22581</v>
       </c>
       <c r="K92" t="n">
-        <v>1.75122</v>
+        <v>1.75145</v>
       </c>
       <c r="L92" t="inlineStr">
         <is>
@@ -4444,7 +4444,7 @@
         <v>-0.9389999999999999</v>
       </c>
       <c r="K93" t="n">
-        <v>1.48794</v>
+        <v>1.47512</v>
       </c>
       <c r="L93" t="inlineStr">
         <is>
@@ -4487,7 +4487,7 @@
         <v>-1.3879</v>
       </c>
       <c r="K94" t="n">
-        <v>1.26566</v>
+        <v>1.25288</v>
       </c>
       <c r="L94" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
         <v>-1.27398</v>
       </c>
       <c r="K96" t="n">
-        <v>1.20819</v>
+        <v>1.22106</v>
       </c>
       <c r="L96" t="inlineStr">
         <is>
@@ -4702,7 +4702,7 @@
         <v>-2.02135</v>
       </c>
       <c r="K99" t="n">
-        <v>1.96401</v>
+        <v>1.97694</v>
       </c>
       <c r="L99" t="inlineStr">
         <is>
@@ -4788,7 +4788,7 @@
         <v>-1.59591</v>
       </c>
       <c r="K101" t="n">
-        <v>2.3003</v>
+        <v>2.30059</v>
       </c>
       <c r="L101" t="inlineStr">
         <is>
@@ -4874,7 +4874,7 @@
         <v>-0.70105</v>
       </c>
       <c r="K103" t="n">
-        <v>3.12263</v>
+        <v>3.13567</v>
       </c>
       <c r="L103" t="inlineStr">
         <is>
@@ -4917,7 +4917,7 @@
         <v>-1.63677</v>
       </c>
       <c r="K104" t="n">
-        <v>3.4042</v>
+        <v>3.41729</v>
       </c>
       <c r="L104" t="inlineStr">
         <is>
@@ -4960,7 +4960,7 @@
         <v>-1.31027</v>
       </c>
       <c r="K105" t="n">
-        <v>3.72851</v>
+        <v>3.72898</v>
       </c>
       <c r="L105" t="inlineStr">
         <is>
@@ -5003,7 +5003,7 @@
         <v>-1.71536</v>
       </c>
       <c r="K106" t="n">
-        <v>4.01464</v>
+        <v>4.01515</v>
       </c>
       <c r="L106" t="inlineStr">
         <is>
@@ -5089,7 +5089,7 @@
         <v>1.6503</v>
       </c>
       <c r="K108" t="n">
-        <v>4.39809</v>
+        <v>4.38552</v>
       </c>
       <c r="L108" t="inlineStr">
         <is>
@@ -5261,7 +5261,7 @@
         <v>1.75485</v>
       </c>
       <c r="K112" t="n">
-        <v>4.54264</v>
+        <v>4.53026</v>
       </c>
       <c r="L112" t="inlineStr">
         <is>
@@ -5304,7 +5304,7 @@
         <v>2.68801</v>
       </c>
       <c r="K113" t="n">
-        <v>4.54658</v>
+        <v>4.5595</v>
       </c>
       <c r="L113" t="inlineStr">
         <is>
@@ -5347,7 +5347,7 @@
         <v>2.87432</v>
       </c>
       <c r="K114" t="n">
-        <v>4.57903</v>
+        <v>4.56672</v>
       </c>
       <c r="L114" t="inlineStr">
         <is>
@@ -5433,7 +5433,7 @@
         <v>3.93853</v>
       </c>
       <c r="K116" t="n">
-        <v>4.5894</v>
+        <v>4.57716</v>
       </c>
       <c r="L116" t="inlineStr">
         <is>
@@ -5476,7 +5476,7 @@
         <v>3.90911</v>
       </c>
       <c r="K117" t="n">
-        <v>4.53272</v>
+        <v>4.53327</v>
       </c>
       <c r="L117" t="inlineStr">
         <is>
@@ -5519,7 +5519,7 @@
         <v>5.25938</v>
       </c>
       <c r="K118" t="n">
-        <v>4.33305</v>
+        <v>4.34571</v>
       </c>
       <c r="L118" t="inlineStr">
         <is>
@@ -5562,7 +5562,7 @@
         <v>3.59819</v>
       </c>
       <c r="K119" t="n">
-        <v>4.29055</v>
+        <v>4.27846</v>
       </c>
       <c r="L119" t="inlineStr">
         <is>
@@ -5605,7 +5605,7 @@
         <v>1.88625</v>
       </c>
       <c r="K120" t="n">
-        <v>4.02022</v>
+        <v>4.03274</v>
       </c>
       <c r="L120" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
         <v>1.4736</v>
       </c>
       <c r="K121" t="n">
-        <v>3.51591</v>
+        <v>3.50395</v>
       </c>
       <c r="L121" t="inlineStr">
         <is>
@@ -5691,7 +5691,7 @@
         <v>3.3177</v>
       </c>
       <c r="K122" t="n">
-        <v>2.90615</v>
+        <v>2.89424</v>
       </c>
       <c r="L122" t="inlineStr">
         <is>
@@ -5777,7 +5777,7 @@
         <v>2.21633</v>
       </c>
       <c r="K124" t="n">
-        <v>2.36798</v>
+        <v>2.38011</v>
       </c>
       <c r="L124" t="inlineStr">
         <is>
@@ -5863,7 +5863,7 @@
         <v>0.27475</v>
       </c>
       <c r="K126" t="n">
-        <v>1.95386</v>
+        <v>1.95409</v>
       </c>
       <c r="L126" t="inlineStr">
         <is>
@@ -5949,7 +5949,7 @@
         <v>-0.16223</v>
       </c>
       <c r="K128" t="n">
-        <v>1.63819</v>
+        <v>1.65009</v>
       </c>
       <c r="L128" t="inlineStr">
         <is>
@@ -5992,7 +5992,7 @@
         <v>0.60939</v>
       </c>
       <c r="K129" t="n">
-        <v>1.13067</v>
+        <v>1.14246</v>
       </c>
       <c r="L129" t="inlineStr">
         <is>
@@ -6078,7 +6078,7 @@
         <v>-6.44729</v>
       </c>
       <c r="K131" t="n">
-        <v>0.35925</v>
+        <v>0.37089</v>
       </c>
       <c r="L131" t="inlineStr">
         <is>
@@ -6164,7 +6164,7 @@
         <v>-7.8633</v>
       </c>
       <c r="K133" t="n">
-        <v>-0.06932000000000001</v>
+        <v>-0.05777</v>
       </c>
       <c r="L133" t="inlineStr">
         <is>
@@ -6207,7 +6207,7 @@
         <v>-7.87933</v>
       </c>
       <c r="K134" t="n">
-        <v>0.53241</v>
+        <v>0.53247</v>
       </c>
       <c r="L134" t="inlineStr">
         <is>
@@ -6293,7 +6293,7 @@
         <v>-7.1485</v>
       </c>
       <c r="K136" t="n">
-        <v>1.04094</v>
+        <v>1.02938</v>
       </c>
       <c r="L136" t="inlineStr">
         <is>
@@ -6379,7 +6379,7 @@
         <v>-6.62404</v>
       </c>
       <c r="K138" t="n">
-        <v>1.68552</v>
+        <v>1.69726</v>
       </c>
       <c r="L138" t="inlineStr">
         <is>
@@ -6551,7 +6551,7 @@
         <v>-5.4778</v>
       </c>
       <c r="K142" t="n">
-        <v>2.83901</v>
+        <v>2.82747</v>
       </c>
       <c r="L142" t="inlineStr">
         <is>
@@ -6594,7 +6594,7 @@
         <v>-0.53771</v>
       </c>
       <c r="K143" t="n">
-        <v>3.30254</v>
+        <v>3.29099</v>
       </c>
       <c r="L143" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
         <v>3.67652</v>
       </c>
       <c r="K146" t="n">
-        <v>3.75317</v>
+        <v>3.76511</v>
       </c>
       <c r="L146" t="inlineStr">
         <is>
@@ -6809,7 +6809,7 @@
         <v>2.77778</v>
       </c>
       <c r="K148" t="n">
-        <v>3.17079</v>
+        <v>3.1826</v>
       </c>
       <c r="L148" t="inlineStr">
         <is>
@@ -6852,7 +6852,7 @@
         <v>2.01723</v>
       </c>
       <c r="K149" t="n">
-        <v>2.658</v>
+        <v>2.64659</v>
       </c>
       <c r="L149" t="inlineStr">
         <is>
@@ -7067,7 +7067,7 @@
         <v>1.1216</v>
       </c>
       <c r="K154" t="n">
-        <v>1.4252</v>
+        <v>1.42536</v>
       </c>
       <c r="L154" t="inlineStr">
         <is>
@@ -7110,7 +7110,7 @@
         <v>2.58983</v>
       </c>
       <c r="K155" t="n">
-        <v>1.45316</v>
+        <v>1.46451</v>
       </c>
       <c r="L155" t="inlineStr">
         <is>
@@ -7196,7 +7196,7 @@
         <v>2.43277</v>
       </c>
       <c r="K157" t="n">
-        <v>1.4562</v>
+        <v>1.44509</v>
       </c>
       <c r="L157" t="inlineStr">
         <is>
@@ -7368,7 +7368,7 @@
         <v>2.46817</v>
       </c>
       <c r="K161" t="n">
-        <v>3.11146</v>
+        <v>3.12292</v>
       </c>
       <c r="L161" t="inlineStr">
         <is>
@@ -7497,7 +7497,7 @@
         <v>3.68896</v>
       </c>
       <c r="K164" t="n">
-        <v>4.25839</v>
+        <v>4.24728</v>
       </c>
       <c r="L164" t="inlineStr">
         <is>
@@ -7583,7 +7583,7 @@
         <v>2.53596</v>
       </c>
       <c r="K166" t="n">
-        <v>4.06063</v>
+        <v>4.07215</v>
       </c>
       <c r="L166" t="inlineStr">
         <is>
@@ -7626,7 +7626,7 @@
         <v>3.64588</v>
       </c>
       <c r="K167" t="n">
-        <v>3.83429</v>
+        <v>3.82327</v>
       </c>
       <c r="L167" t="inlineStr">
         <is>
@@ -7712,7 +7712,7 @@
         <v>2.889</v>
       </c>
       <c r="K169" t="n">
-        <v>3.83478</v>
+        <v>3.8352</v>
       </c>
       <c r="L169" t="inlineStr">
         <is>
@@ -7884,7 +7884,7 @@
         <v>2.84697</v>
       </c>
       <c r="K173" t="n">
-        <v>3.55642</v>
+        <v>3.54564</v>
       </c>
       <c r="L173" t="inlineStr">
         <is>
@@ -8013,7 +8013,7 @@
         <v>2.54939</v>
       </c>
       <c r="K176" t="n">
-        <v>2.99669</v>
+        <v>3.00768</v>
       </c>
       <c r="L176" t="inlineStr">
         <is>
@@ -8142,7 +8142,7 @@
         <v>2.50148</v>
       </c>
       <c r="K179" t="n">
-        <v>2.92869</v>
+        <v>2.93962</v>
       </c>
       <c r="L179" t="inlineStr">
         <is>
@@ -8228,7 +8228,7 @@
         <v>1.81115</v>
       </c>
       <c r="K181" t="n">
-        <v>2.91231</v>
+        <v>2.92317</v>
       </c>
       <c r="L181" t="inlineStr">
         <is>
@@ -8400,7 +8400,7 @@
         <v>1.47007</v>
       </c>
       <c r="K185" t="n">
-        <v>1.87324</v>
+        <v>1.88385</v>
       </c>
       <c r="L185" t="inlineStr">
         <is>
@@ -9518,7 +9518,7 @@
         <v>-3.18673</v>
       </c>
       <c r="K211" t="n">
-        <v>-1.73826</v>
+        <v>-1.72827</v>
       </c>
       <c r="L211" t="inlineStr">
         <is>
@@ -10034,7 +10034,7 @@
         <v>-8.699949999999999</v>
       </c>
       <c r="K223" t="n">
-        <v>-6.07971</v>
+        <v>-6.08925</v>
       </c>
       <c r="L223" t="inlineStr">
         <is>
@@ -10249,7 +10249,7 @@
         <v>-4.18348</v>
       </c>
       <c r="K228" t="n">
-        <v>-3.35289</v>
+        <v>-3.34241</v>
       </c>
       <c r="L228" t="inlineStr">
         <is>
@@ -10292,7 +10292,7 @@
         <v>-4.2065</v>
       </c>
       <c r="K229" t="n">
-        <v>-2.5132</v>
+        <v>-2.50264</v>
       </c>
       <c r="L229" t="inlineStr">
         <is>
@@ -10550,7 +10550,7 @@
         <v>-1.35654</v>
       </c>
       <c r="K235" t="n">
-        <v>1.19073</v>
+        <v>1.20156</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -10636,7 +10636,7 @@
         <v>-0.25725</v>
       </c>
       <c r="K237" t="n">
-        <v>1.59315</v>
+        <v>1.60399</v>
       </c>
       <c r="L237" t="inlineStr">
         <is>
@@ -10765,7 +10765,7 @@
         <v>1.67509</v>
       </c>
       <c r="K240" t="n">
-        <v>1.84302</v>
+        <v>1.84282</v>
       </c>
       <c r="L240" t="inlineStr">
         <is>
@@ -10808,7 +10808,7 @@
         <v>2.18762</v>
       </c>
       <c r="K241" t="n">
-        <v>1.83059</v>
+        <v>1.83039</v>
       </c>
       <c r="L241" t="inlineStr">
         <is>
@@ -10894,7 +10894,7 @@
         <v>2.64173</v>
       </c>
       <c r="K243" t="n">
-        <v>2.11755</v>
+        <v>2.12835</v>
       </c>
       <c r="L243" t="inlineStr">
         <is>
@@ -11066,7 +11066,7 @@
         <v>3.46116</v>
       </c>
       <c r="K247" t="n">
-        <v>1.06975</v>
+        <v>1.05894</v>
       </c>
       <c r="L247" t="inlineStr">
         <is>
@@ -11152,7 +11152,7 @@
         <v>4.28998</v>
       </c>
       <c r="K249" t="n">
-        <v>0.82142</v>
+        <v>0.81067</v>
       </c>
       <c r="L249" t="inlineStr">
         <is>
@@ -11195,7 +11195,7 @@
         <v>5.36587</v>
       </c>
       <c r="K250" t="n">
-        <v>1.08939</v>
+        <v>1.10007</v>
       </c>
       <c r="L250" t="inlineStr">
         <is>
@@ -11238,7 +11238,7 @@
         <v>4.6915</v>
       </c>
       <c r="K251" t="n">
-        <v>1.32238</v>
+        <v>1.33305</v>
       </c>
       <c r="L251" t="inlineStr">
         <is>
@@ -11281,7 +11281,7 @@
         <v>4.78751</v>
       </c>
       <c r="K252" t="n">
-        <v>1.54354</v>
+        <v>1.53273</v>
       </c>
       <c r="L252" t="inlineStr">
         <is>
@@ -11324,7 +11324,7 @@
         <v>4.94873</v>
       </c>
       <c r="K253" t="n">
-        <v>2.12743</v>
+        <v>2.11657</v>
       </c>
       <c r="L253" t="inlineStr">
         <is>
@@ -11367,7 +11367,7 @@
         <v>5.60819</v>
       </c>
       <c r="K254" t="n">
-        <v>2.03498</v>
+        <v>2.04557</v>
       </c>
       <c r="L254" t="inlineStr">
         <is>
@@ -11410,7 +11410,7 @@
         <v>5.94848</v>
       </c>
       <c r="K255" t="n">
-        <v>2.40161</v>
+        <v>2.39078</v>
       </c>
       <c r="L255" t="inlineStr">
         <is>
@@ -11668,7 +11668,7 @@
         <v>5.46892</v>
       </c>
       <c r="K261" t="n">
-        <v>5.34335</v>
+        <v>5.35393</v>
       </c>
       <c r="L261" t="inlineStr">
         <is>
@@ -11711,7 +11711,7 @@
         <v>4.06068</v>
       </c>
       <c r="K262" t="n">
-        <v>5.82145</v>
+        <v>5.81027</v>
       </c>
       <c r="L262" t="inlineStr">
         <is>
@@ -11754,7 +11754,7 @@
         <v>3.98664</v>
       </c>
       <c r="K263" t="n">
-        <v>5.86254</v>
+        <v>5.86192</v>
       </c>
       <c r="L263" t="inlineStr">
         <is>
@@ -11797,7 +11797,7 @@
         <v>3.80942</v>
       </c>
       <c r="K264" t="n">
-        <v>5.93354</v>
+        <v>5.94402</v>
       </c>
       <c r="L264" t="inlineStr">
         <is>
@@ -11883,7 +11883,7 @@
         <v>2.87385</v>
       </c>
       <c r="K266" t="n">
-        <v>5.64039</v>
+        <v>5.62941</v>
       </c>
       <c r="L266" t="inlineStr">
         <is>
@@ -11969,7 +11969,7 @@
         <v>2.18501</v>
       </c>
       <c r="K268" t="n">
-        <v>5.869</v>
+        <v>5.87932</v>
       </c>
       <c r="L268" t="inlineStr">
         <is>
@@ -12012,7 +12012,7 @@
         <v>2.61295</v>
       </c>
       <c r="K269" t="n">
-        <v>5.81288</v>
+        <v>5.82315</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
@@ -12055,7 +12055,7 @@
         <v>2.24409</v>
       </c>
       <c r="K270" t="n">
-        <v>5.57374</v>
+        <v>5.58396</v>
       </c>
       <c r="L270" t="inlineStr">
         <is>
@@ -12184,7 +12184,7 @@
         <v>2.87077</v>
       </c>
       <c r="K273" t="n">
-        <v>4.37927</v>
+        <v>4.36879</v>
       </c>
       <c r="L273" t="inlineStr">
         <is>
@@ -12270,7 +12270,7 @@
         <v>2.59061</v>
       </c>
       <c r="K275" t="n">
-        <v>3.37045</v>
+        <v>3.36017</v>
       </c>
       <c r="L275" t="inlineStr">
         <is>
@@ -12313,7 +12313,7 @@
         <v>2.64213</v>
       </c>
       <c r="K276" t="n">
-        <v>2.99852</v>
+        <v>2.99822</v>
       </c>
       <c r="L276" t="inlineStr">
         <is>
@@ -12399,7 +12399,7 @@
         <v>3.57057</v>
       </c>
       <c r="K278" t="n">
-        <v>2.88102</v>
+        <v>2.89086</v>
       </c>
       <c r="L278" t="inlineStr">
         <is>
@@ -12442,7 +12442,7 @@
         <v>3.10631</v>
       </c>
       <c r="K279" t="n">
-        <v>2.72914</v>
+        <v>2.73892</v>
       </c>
       <c r="L279" t="inlineStr">
         <is>
@@ -12485,7 +12485,7 @@
         <v>3.13352</v>
       </c>
       <c r="K280" t="n">
-        <v>2.72798</v>
+        <v>2.71797</v>
       </c>
       <c r="L280" t="inlineStr">
         <is>
@@ -12528,7 +12528,7 @@
         <v>2.52939</v>
       </c>
       <c r="K281" t="n">
-        <v>2.48471</v>
+        <v>2.47477</v>
       </c>
       <c r="L281" t="inlineStr">
         <is>
@@ -12571,7 +12571,7 @@
         <v>2.46755</v>
       </c>
       <c r="K282" t="n">
-        <v>2.7027</v>
+        <v>2.69275</v>
       </c>
       <c r="L282" t="inlineStr">
         <is>
@@ -12614,7 +12614,7 @@
         <v>1.70802</v>
       </c>
       <c r="K283" t="n">
-        <v>2.45103</v>
+        <v>2.46068</v>
       </c>
       <c r="L283" t="inlineStr">
         <is>
@@ -12700,7 +12700,7 @@
         <v>0.5518</v>
       </c>
       <c r="K285" t="n">
-        <v>2.99269</v>
+        <v>3.00231</v>
       </c>
       <c r="L285" t="inlineStr">
         <is>
@@ -12829,7 +12829,7 @@
         <v>0.5296999999999999</v>
       </c>
       <c r="K288" t="n">
-        <v>3.8432</v>
+        <v>3.84283</v>
       </c>
       <c r="L288" t="inlineStr">
         <is>
@@ -12915,7 +12915,7 @@
         <v>-0.04054</v>
       </c>
       <c r="K290" t="n">
-        <v>3.83255</v>
+        <v>3.82263</v>
       </c>
       <c r="L290" t="inlineStr">
         <is>
@@ -12958,7 +12958,7 @@
         <v>-0.23617</v>
       </c>
       <c r="K291" t="n">
-        <v>3.85641</v>
+        <v>3.84652</v>
       </c>
       <c r="L291" t="inlineStr">
         <is>
@@ -13001,7 +13001,7 @@
         <v>-0.7377899999999999</v>
       </c>
       <c r="K292" t="n">
-        <v>3.61343</v>
+        <v>3.62291</v>
       </c>
       <c r="L292" t="inlineStr">
         <is>
@@ -13044,7 +13044,7 @@
         <v>-0.52172</v>
       </c>
       <c r="K293" t="n">
-        <v>3.87347</v>
+        <v>3.88294</v>
       </c>
       <c r="L293" t="inlineStr">
         <is>
@@ -13087,7 +13087,7 @@
         <v>-0.8229</v>
       </c>
       <c r="K294" t="n">
-        <v>3.87663</v>
+        <v>3.88606</v>
       </c>
       <c r="L294" t="inlineStr">
         <is>
@@ -13130,7 +13130,7 @@
         <v>-0.05906</v>
       </c>
       <c r="K295" t="n">
-        <v>4.15372</v>
+        <v>4.14391</v>
       </c>
       <c r="L295" t="inlineStr">
         <is>
@@ -13173,7 +13173,7 @@
         <v>0.27712</v>
       </c>
       <c r="K296" t="n">
-        <v>4.17527</v>
+        <v>4.18465</v>
       </c>
       <c r="L296" t="inlineStr">
         <is>
@@ -13216,7 +13216,7 @@
         <v>0.31426</v>
       </c>
       <c r="K297" t="n">
-        <v>3.95216</v>
+        <v>3.95179</v>
       </c>
       <c r="L297" t="inlineStr">
         <is>
@@ -13345,7 +13345,7 @@
         <v>1.00172</v>
       </c>
       <c r="K300" t="n">
-        <v>3.58993</v>
+        <v>3.58035</v>
       </c>
       <c r="L300" t="inlineStr">
         <is>
@@ -13388,7 +13388,7 @@
         <v>1.95501</v>
       </c>
       <c r="K301" t="n">
-        <v>3.94749</v>
+        <v>3.95673</v>
       </c>
       <c r="L301" t="inlineStr">
         <is>
@@ -13431,7 +13431,7 @@
         <v>1.47719</v>
       </c>
       <c r="K302" t="n">
-        <v>3.58063</v>
+        <v>3.58984</v>
       </c>
       <c r="L302" t="inlineStr">
         <is>
@@ -13517,7 +13517,7 @@
         <v>2.73019</v>
       </c>
       <c r="K304" t="n">
-        <v>3.55149</v>
+        <v>3.55116</v>
       </c>
       <c r="L304" t="inlineStr">
         <is>
@@ -13560,7 +13560,7 @@
         <v>2.50477</v>
       </c>
       <c r="K305" t="n">
-        <v>3.30051</v>
+        <v>3.30021</v>
       </c>
       <c r="L305" t="inlineStr">
         <is>
@@ -13603,7 +13603,7 @@
         <v>2.97813</v>
       </c>
       <c r="K306" t="n">
-        <v>3.0237</v>
+        <v>3.02342</v>
       </c>
       <c r="L306" t="inlineStr">
         <is>
@@ -13646,7 +13646,7 @@
         <v>3.47011</v>
       </c>
       <c r="K307" t="n">
-        <v>2.72201</v>
+        <v>2.73105</v>
       </c>
       <c r="L307" t="inlineStr">
         <is>
@@ -13689,7 +13689,7 @@
         <v>3.01415</v>
       </c>
       <c r="K308" t="n">
-        <v>2.738</v>
+        <v>2.73775</v>
       </c>
       <c r="L308" t="inlineStr">
         <is>
@@ -13732,7 +13732,7 @@
         <v>3.06809</v>
       </c>
       <c r="K309" t="n">
-        <v>2.73234</v>
+        <v>2.73209</v>
       </c>
       <c r="L309" t="inlineStr">
         <is>
@@ -13775,7 +13775,7 @@
         <v>2.6111</v>
       </c>
       <c r="K310" t="n">
-        <v>2.76832</v>
+        <v>2.77728</v>
       </c>
       <c r="L310" t="inlineStr">
         <is>
@@ -13818,7 +13818,7 @@
         <v>2.99353</v>
       </c>
       <c r="K311" t="n">
-        <v>2.69134</v>
+        <v>2.70029</v>
       </c>
       <c r="L311" t="inlineStr">
         <is>
@@ -13904,7 +13904,7 @@
         <v>2.39374</v>
       </c>
       <c r="K313" t="n">
-        <v>2.926</v>
+        <v>2.92574</v>
       </c>
       <c r="L313" t="inlineStr">
         <is>
@@ -13947,7 +13947,7 @@
         <v>1.92627</v>
       </c>
       <c r="K314" t="n">
-        <v>3.01253</v>
+        <v>3.01226</v>
       </c>
       <c r="L314" t="inlineStr">
         <is>
@@ -14033,7 +14033,7 @@
         <v>2.62675</v>
       </c>
       <c r="K316" t="n">
-        <v>3.03191</v>
+        <v>3.03164</v>
       </c>
       <c r="L316" t="inlineStr">
         <is>
@@ -14076,7 +14076,7 @@
         <v>3.43649</v>
       </c>
       <c r="K317" t="n">
-        <v>3.27449</v>
+        <v>3.2742</v>
       </c>
       <c r="L317" t="inlineStr">
         <is>
@@ -14119,7 +14119,7 @@
         <v>3.3741</v>
       </c>
       <c r="K318" t="n">
-        <v>3.52547</v>
+        <v>3.52516</v>
       </c>
       <c r="L318" t="inlineStr">
         <is>
@@ -14162,7 +14162,7 @@
         <v>3.14975</v>
       </c>
       <c r="K319" t="n">
-        <v>3.82076</v>
+        <v>3.82042</v>
       </c>
       <c r="L319" t="inlineStr">
         <is>
@@ -14205,7 +14205,7 @@
         <v>3.12855</v>
       </c>
       <c r="K320" t="n">
-        <v>3.52415</v>
+        <v>3.52384</v>
       </c>
       <c r="L320" t="inlineStr">
         <is>
@@ -14248,7 +14248,7 @@
         <v>3.1808</v>
       </c>
       <c r="K321" t="n">
-        <v>3.64829</v>
+        <v>3.63923</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -14291,7 +14291,7 @@
         <v>3.7925</v>
       </c>
       <c r="K322" t="n">
-        <v>3.73987</v>
+        <v>3.73954</v>
       </c>
       <c r="L322" t="inlineStr">
         <is>
@@ -14334,7 +14334,7 @@
         <v>3.92538</v>
       </c>
       <c r="K323" t="n">
-        <v>3.76143</v>
+        <v>3.7611</v>
       </c>
       <c r="L323" t="inlineStr">
         <is>
@@ -14377,7 +14377,7 @@
         <v>3.68468</v>
       </c>
       <c r="K324" t="n">
-        <v>3.45157</v>
+        <v>3.46024</v>
       </c>
       <c r="L324" t="inlineStr">
         <is>
@@ -14420,7 +14420,7 @@
         <v>3.30291</v>
       </c>
       <c r="K325" t="n">
-        <v>3.22302</v>
+        <v>3.22274</v>
       </c>
       <c r="L325" t="inlineStr">
         <is>
@@ -14463,7 +14463,7 @@
         <v>2.86511</v>
       </c>
       <c r="K326" t="n">
-        <v>2.9158</v>
+        <v>2.91555</v>
       </c>
       <c r="L326" t="inlineStr">
         <is>
@@ -14506,7 +14506,7 @@
         <v>2.05802</v>
       </c>
       <c r="K327" t="n">
-        <v>2.63814</v>
+        <v>2.64673</v>
       </c>
       <c r="L327" t="inlineStr">
         <is>
@@ -14549,7 +14549,7 @@
         <v>1.82602</v>
       </c>
       <c r="K328" t="n">
-        <v>2.3593</v>
+        <v>2.3591</v>
       </c>
       <c r="L328" t="inlineStr">
         <is>
@@ -14592,7 +14592,7 @@
         <v>1.16177</v>
       </c>
       <c r="K329" t="n">
-        <v>2.05965</v>
+        <v>2.05948</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -14635,7 +14635,7 @@
         <v>1.15674</v>
       </c>
       <c r="K330" t="n">
-        <v>1.53244</v>
+        <v>1.53231</v>
       </c>
       <c r="L330" t="inlineStr">
         <is>
@@ -14678,7 +14678,7 @@
         <v>0.72941</v>
       </c>
       <c r="K331" t="n">
-        <v>1.00907</v>
+        <v>1.00899</v>
       </c>
       <c r="L331" t="inlineStr">
         <is>
@@ -14721,7 +14721,7 @@
         <v>1.13298</v>
       </c>
       <c r="K332" t="n">
-        <v>0.9569</v>
+        <v>0.94835</v>
       </c>
       <c r="L332" t="inlineStr">
         <is>
@@ -14764,7 +14764,7 @@
         <v>1.19602</v>
       </c>
       <c r="K333" t="n">
-        <v>0.54022</v>
+        <v>0.54866</v>
       </c>
       <c r="L333" t="inlineStr">
         <is>
@@ -14893,7 +14893,7 @@
         <v>-2.43287</v>
       </c>
       <c r="K336" t="n">
-        <v>-0.2934</v>
+        <v>-0.29338</v>
       </c>
       <c r="L336" t="inlineStr">
         <is>
@@ -14936,7 +14936,7 @@
         <v>2.74486</v>
       </c>
       <c r="K337" t="n">
-        <v>-0.32647</v>
+        <v>-0.32644</v>
       </c>
       <c r="L337" t="inlineStr">
         <is>
@@ -14979,7 +14979,7 @@
         <v>-0.53278</v>
       </c>
       <c r="K338" t="n">
-        <v>-0.36044</v>
+        <v>-0.36041</v>
       </c>
       <c r="L338" t="inlineStr">
         <is>
@@ -15022,7 +15022,7 @@
         <v>-0.09285</v>
       </c>
       <c r="K339" t="n">
-        <v>-0.10884</v>
+        <v>-0.10883</v>
       </c>
       <c r="L339" t="inlineStr">
         <is>
@@ -15065,7 +15065,7 @@
         <v>-0.52616</v>
       </c>
       <c r="K340" t="n">
-        <v>0.14249</v>
+        <v>0.14247</v>
       </c>
       <c r="L340" t="inlineStr">
         <is>
@@ -15108,7 +15108,7 @@
         <v>-1.22507</v>
       </c>
       <c r="K341" t="n">
-        <v>0.40194</v>
+        <v>0.40191</v>
       </c>
       <c r="L341" t="inlineStr">
         <is>
@@ -15151,7 +15151,7 @@
         <v>-1.44273</v>
       </c>
       <c r="K342" t="n">
-        <v>0.69596</v>
+        <v>0.6959</v>
       </c>
       <c r="L342" t="inlineStr">
         <is>
@@ -15194,7 +15194,7 @@
         <v>-1.09171</v>
       </c>
       <c r="K343" t="n">
-        <v>1.1501</v>
+        <v>1.15</v>
       </c>
       <c r="L343" t="inlineStr">
         <is>
@@ -15237,7 +15237,7 @@
         <v>-0.75704</v>
       </c>
       <c r="K344" t="n">
-        <v>1.20785</v>
+        <v>1.21624</v>
       </c>
       <c r="L344" t="inlineStr">
         <is>
@@ -15280,7 +15280,7 @@
         <v>-0.69376</v>
       </c>
       <c r="K345" t="n">
-        <v>1.66233</v>
+        <v>1.66219</v>
       </c>
       <c r="L345" t="inlineStr">
         <is>
@@ -15323,7 +15323,7 @@
         <v>-0.13945</v>
       </c>
       <c r="K346" t="n">
-        <v>2.05163</v>
+        <v>2.05145</v>
       </c>
       <c r="L346" t="inlineStr">
         <is>
@@ -15366,7 +15366,7 @@
         <v>-1.0381</v>
       </c>
       <c r="K347" t="n">
-        <v>2.04082</v>
+        <v>2.04064</v>
       </c>
       <c r="L347" t="inlineStr">
         <is>
@@ -15409,7 +15409,7 @@
         <v>2.99158</v>
       </c>
       <c r="K348" t="n">
-        <v>2.53069</v>
+        <v>2.53047</v>
       </c>
       <c r="L348" t="inlineStr">
         <is>
@@ -15452,7 +15452,7 @@
         <v>-1.39386</v>
       </c>
       <c r="K349" t="n">
-        <v>2.79667</v>
+        <v>2.79644</v>
       </c>
       <c r="L349" t="inlineStr">
         <is>
@@ -15495,7 +15495,7 @@
         <v>2.56005</v>
       </c>
       <c r="K350" t="n">
-        <v>3.17153</v>
+        <v>3.17127</v>
       </c>
       <c r="L350" t="inlineStr">
         <is>
@@ -15538,7 +15538,7 @@
         <v>1.78134</v>
       </c>
       <c r="K351" t="n">
-        <v>2.90839</v>
+        <v>2.90815</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -15581,7 +15581,7 @@
         <v>1.56742</v>
       </c>
       <c r="K352" t="n">
-        <v>3.0298</v>
+        <v>3.02954</v>
       </c>
       <c r="L352" t="inlineStr">
         <is>
@@ -15624,7 +15624,7 @@
         <v>-49.2774</v>
       </c>
       <c r="K353" t="n">
-        <v>-38.87406</v>
+        <v>-38.87916</v>
       </c>
       <c r="L353" t="inlineStr">
         <is>
@@ -15667,7 +15667,7 @@
         <v>-69.48389</v>
       </c>
       <c r="K354" t="n">
-        <v>-38.42118</v>
+        <v>-38.41799</v>
       </c>
       <c r="L354" t="inlineStr">
         <is>
@@ -15710,7 +15710,7 @@
         <v>-70.07268000000001</v>
       </c>
       <c r="K355" t="n">
-        <v>-33.27247</v>
+        <v>-33.26971</v>
       </c>
       <c r="L355" t="inlineStr">
         <is>
@@ -15753,7 +15753,7 @@
         <v>-74.73842</v>
       </c>
       <c r="K356" t="n">
-        <v>-30.14255</v>
+        <v>-30.14005</v>
       </c>
       <c r="L356" t="inlineStr">
         <is>
@@ -15796,7 +15796,7 @@
         <v>-74.86150000000001</v>
       </c>
       <c r="K357" t="n">
-        <v>-25.53473</v>
+        <v>-25.53262</v>
       </c>
       <c r="L357" t="inlineStr">
         <is>
@@ -15839,7 +15839,7 @@
         <v>-76.53857000000001</v>
       </c>
       <c r="K358" t="n">
-        <v>-26.06081</v>
+        <v>-26.05866</v>
       </c>
       <c r="L358" t="inlineStr">
         <is>
@@ -15882,7 +15882,7 @@
         <v>-66.67775</v>
       </c>
       <c r="K359" t="n">
-        <v>-22.15638</v>
+        <v>-22.15456</v>
       </c>
       <c r="L359" t="inlineStr">
         <is>
@@ -15925,7 +15925,7 @@
         <v>-56.85972</v>
       </c>
       <c r="K360" t="n">
-        <v>-20.3936</v>
+        <v>-20.39193</v>
       </c>
       <c r="L360" t="inlineStr">
         <is>
@@ -15968,7 +15968,7 @@
         <v>-53.25212</v>
       </c>
       <c r="K361" t="n">
-        <v>-19.73039</v>
+        <v>-19.72878</v>
       </c>
       <c r="L361" t="inlineStr">
         <is>

</xml_diff>